<commit_message>
added EFR to logical model
</commit_message>
<xml_diff>
--- a/StructureDefinition-VunsPatient.xlsx
+++ b/StructureDefinition-VunsPatient.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-08-04T16:28:32+02:00</t>
+    <t>2025-08-18T11:20:46+02:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Profil pour un Patient enrôlé dans le cadre du projet Vers Un Souffle Nouveau</t>
+    <t>Profile for patient enrolled in the 'Vers Un Souffle Nouveau' project</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -1183,7 +1183,7 @@
   </si>
   <si>
     <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-PhoneNumber:Format des numéros de téléphone {matches('\\d+')}</t>
+PhoneNumber:Phone number format {matches('\\d+')}</t>
   </si>
   <si>
     <t>./url</t>
@@ -1278,7 +1278,7 @@
   </si>
   <si>
     <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-Email:Format des emails {matches('\\S+@\\S+\\.\\S+')}</t>
+Email:Email format {matches('\\S+@\\S+\\.\\S+')}</t>
   </si>
   <si>
     <t>Patient.telecom:email.use</t>

</xml_diff>